<commit_message>
Fix PDF parameter parsing and normalize hematology units
</commit_message>
<xml_diff>
--- a/ml/reports/evaluation/test_predictions.xlsx
+++ b/ml/reports/evaluation/test_predictions.xlsx
@@ -19904,7 +19904,7 @@
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>0.006156704567109193</v>
+        <v>0.006156704567109191</v>
       </c>
     </row>
     <row r="48">
@@ -22289,7 +22289,7 @@
         <v>1</v>
       </c>
       <c r="M100" t="n">
-        <v>0.3974722222222222</v>
+        <v>0.3974722222222223</v>
       </c>
     </row>
     <row r="101">
@@ -22559,7 +22559,7 @@
         <v>1</v>
       </c>
       <c r="M106" t="n">
-        <v>0.07786858041056398</v>
+        <v>0.07786858041056396</v>
       </c>
     </row>
     <row r="107">

</xml_diff>